<commit_message>
feat: implement download links and transmittal email logic
</commit_message>
<xml_diff>
--- a/tasks.xlsx
+++ b/tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marlen\PycharmProjects\edms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{89748A09-D0DF-4FBA-B33B-A38FC0C5E16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE4E384B-A43F-4949-BD32-F75FBBA5BCE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B00D21D6-71DC-4FDB-9CB6-65DCE6EA6F08}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="26">
   <si>
     <t>Advance search button (search document by tag or text)</t>
   </si>
@@ -112,6 +112,12 @@
   </si>
   <si>
     <t>нужно обсудить</t>
+  </si>
+  <si>
+    <t>+</t>
+  </si>
+  <si>
+    <t>вручную на транмиттале</t>
   </si>
 </sst>
 </file>
@@ -488,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{988267C0-7ACC-420D-BB4D-9DDC7B21EEE5}">
-  <dimension ref="I6:J25"/>
+  <dimension ref="H6:J25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="9" max="9" width="72.28515625" bestFit="1" customWidth="1"/>
@@ -580,7 +586,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>24</v>
+      </c>
       <c r="I17" t="s">
         <v>1</v>
       </c>
@@ -588,7 +597,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="18" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>24</v>
+      </c>
       <c r="I18" t="s">
         <v>2</v>
       </c>
@@ -596,7 +608,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>24</v>
+      </c>
       <c r="I19" t="s">
         <v>3</v>
       </c>
@@ -604,7 +619,10 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>24</v>
+      </c>
       <c r="I20" t="s">
         <v>4</v>
       </c>
@@ -612,27 +630,36 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="8:10" x14ac:dyDescent="0.25">
       <c r="I21" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H22" t="s">
+        <v>24</v>
+      </c>
       <c r="I22" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="23" spans="9:10" x14ac:dyDescent="0.25">
+      <c r="J22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="8:10" x14ac:dyDescent="0.25">
       <c r="I23" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="8:10" x14ac:dyDescent="0.25">
       <c r="I24" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="25" spans="9:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="8:10" x14ac:dyDescent="0.25">
+      <c r="H25" t="s">
+        <v>24</v>
+      </c>
       <c r="I25" t="s">
         <v>19</v>
       </c>

</xml_diff>